<commit_message>
replacing "grinded" with "polished"
</commit_message>
<xml_diff>
--- a/doc/examples/resource/resource-alternate.xlsx
+++ b/doc/examples/resource/resource-alternate.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\develop\frepple-community\doc\user-guide\examples\resource\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\jdetaeye\workspace\frepple-community\doc\examples\resource\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C703C26-4B1A-40F8-9EBB-70F0CF714E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23258" windowHeight="12578" tabRatio="813" firstSheet="3" activeTab="12"/>
+    <workbookView xWindow="38400" yWindow="1140" windowWidth="38355" windowHeight="12015" tabRatio="813" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sales order" sheetId="1" r:id="rId1"/>
@@ -111,9 +112,6 @@
     <t>All items</t>
   </si>
   <si>
-    <t>grinded wooden panel</t>
-  </si>
-  <si>
     <t>raw material</t>
   </si>
   <si>
@@ -183,9 +181,6 @@
     <t>Skill</t>
   </si>
   <si>
-    <t>grinded wooden panel supplier</t>
-  </si>
-  <si>
     <t>screw supplier</t>
   </si>
   <si>
@@ -349,16 +344,22 @@
   </si>
   <si>
     <t>plan.webservice</t>
+  </si>
+  <si>
+    <t>polished wooden panel</t>
+  </si>
+  <si>
+    <t>polished wooden panel supplier</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -403,7 +404,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="headerstyle" xfId="1"/>
+    <cellStyle name="headerstyle" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -703,19 +704,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.46484375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.86328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.53125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.53125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -741,7 +742,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -767,7 +768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -793,7 +794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -820,37 +821,37 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1048576"/>
+  <autoFilter ref="A1:H1048576" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.86328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.53125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.86328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.53125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.1328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.1328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.46484375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.86328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>3</v>
@@ -868,36 +869,36 @@
         <v>11</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" t="s">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C2" t="s">
-        <v>58</v>
-      </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
         <v>14</v>
@@ -925,23 +926,23 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M1048576"/>
+  <autoFilter ref="A1:M1048576" xr:uid="{00000000-0009-0000-0000-000009000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.46484375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>6</v>
@@ -950,15 +951,15 @@
         <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
@@ -967,79 +968,79 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>99</v>
       </c>
       <c r="C3">
         <v>-1</v>
       </c>
       <c r="E3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4">
         <v>-10</v>
       </c>
       <c r="E4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C5">
         <v>-4</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1048576"/>
+  <autoFilter ref="A1:E1048576" xr:uid="{00000000-0009-0000-0000-00000A000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.86328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>10</v>
@@ -1048,18 +1049,18 @@
         <v>11</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1068,18 +1069,18 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1088,201 +1089,201 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1048576"/>
+  <autoFilter ref="A1:F1048576" xr:uid="{00000000-0009-0000-0000-00000B000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.46484375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.53125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="136.796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="136.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" t="s">
         <v>66</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>67</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
+      <c r="C3" t="s">
         <v>69</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>70</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B4" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
+      <c r="C4" t="s">
         <v>72</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>73</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B5" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
+      <c r="C5" t="s">
         <v>75</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>76</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B6" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
+      <c r="C6" t="s">
         <v>78</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>79</v>
       </c>
-      <c r="C6" t="s">
+      <c r="B7" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
+      <c r="C7" t="s">
         <v>81</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>82</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>84</v>
       </c>
-      <c r="C8" t="s">
+      <c r="B9" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
+      <c r="C9" t="s">
         <v>86</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>87</v>
       </c>
-      <c r="C9" t="s">
+      <c r="B10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>89</v>
       </c>
-      <c r="B10" t="s">
-        <v>79</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="B11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>91</v>
       </c>
-      <c r="B11" t="s">
-        <v>67</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="B12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>93</v>
       </c>
-      <c r="B12" t="s">
-        <v>67</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="B13" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
+      <c r="C13" t="s">
         <v>95</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>96</v>
       </c>
-      <c r="C13" t="s">
+      <c r="B14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C14" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
-      <c r="A14" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>98</v>
       </c>
-      <c r="B14" t="s">
-        <v>96</v>
-      </c>
-      <c r="C14" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>100</v>
-      </c>
       <c r="B15" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C1048576"/>
+  <autoFilter ref="A1:C1048576" xr:uid="{00000000-0009-0000-0000-00000C000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.46484375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.53125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1299,29 +1300,29 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>99</v>
       </c>
       <c r="B3" t="s">
         <v>20</v>
       </c>
       <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
         <v>22</v>
-      </c>
-      <c r="D3" t="s">
-        <v>23</v>
       </c>
       <c r="E3">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1329,64 +1330,64 @@
         <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4">
         <v>300</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>26</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>27</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E6">
         <v>10</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1048576"/>
+  <autoFilter ref="A1:E1048576" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="10.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1394,58 +1395,58 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B1048576"/>
+  <autoFilter ref="A1:B1048576" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.53125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A1048576"/>
+  <autoFilter ref="A1:A1048576" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="11.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1453,49 +1454,49 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>33</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>34</v>
       </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
+      <c r="C3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>35</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B4" t="s">
         <v>34</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
-      </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1504,15 +1505,15 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -1521,15 +1522,15 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
         <v>33</v>
-      </c>
-      <c r="C6" t="s">
-        <v>34</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1538,15 +1539,15 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
         <v>33</v>
-      </c>
-      <c r="C7" t="s">
-        <v>34</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -1555,183 +1556,183 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>40</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s">
         <v>33</v>
       </c>
-      <c r="C8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" t="s">
-        <v>34</v>
-      </c>
       <c r="D9">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1048576"/>
+  <autoFilter ref="A1:F1048576" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A1048576"/>
+  <autoFilter ref="A1:A1048576" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>36</v>
       </c>
-      <c r="B2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>37</v>
       </c>
-      <c r="B3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>38</v>
       </c>
-      <c r="B4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>39</v>
-      </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C1048576"/>
+  <autoFilter ref="A1:C1048576" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
-      <c r="A3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
-        <v>47</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:A1048576"/>
+  <autoFilter ref="A1:A1048576" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.46484375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.53125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.1328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.1328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -1739,30 +1740,30 @@
         <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E2">
         <v>3000</v>
@@ -1774,15 +1775,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>99</v>
       </c>
       <c r="B3" t="s">
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -1791,15 +1792,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
         <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -1809,7 +1810,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1048576"/>
+  <autoFilter ref="A1:G1048576" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>